<commit_message>
feat: add multi-image support, complete form interaction logic, and initialize automation data structures.
</commit_message>
<xml_diff>
--- a/data/data.xlsx
+++ b/data/data.xlsx
@@ -1,17 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Downloads\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98A5079F-7898-4FA5-8612-685700201418}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="2904" yWindow="1020" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Sheet4" sheetId="1" r:id="rId5"/>
+    <sheet name="Sheet4" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="33">
   <si>
     <t>No</t>
   </si>
@@ -104,22 +113,36 @@
   </si>
   <si>
     <t>Asia | Heidemarie ME6 | 25 SSR Combatant (Inc Dupe) and 5 Partner | 1 Omega and 20 Standard Pull</t>
+  </si>
+  <si>
+    <t>Honkai: Star Rail</t>
+  </si>
+  <si>
+    <t>Asia | 64 Character(Inc Dupe) and 27 Lightcone | Casto E2 | Rate On Pity 40</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color rgb="FF1F1F1F"/>
       <name val="&quot;Google Sans Text&quot;"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -127,40 +150,65 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
-    <border/>
+  <borders count="2">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+  <cellXfs count="5">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -350,23 +398,26 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:E25"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="2" max="2" width="25.25"/>
-    <col customWidth="1" min="3" max="3" width="21.0"/>
-    <col customWidth="1" min="5" max="5" width="85.38"/>
-    <col customWidth="1" min="6" max="6" width="67.5"/>
+    <col min="2" max="2" width="25.21875" customWidth="1"/>
+    <col min="3" max="3" width="21" customWidth="1"/>
+    <col min="5" max="5" width="85.33203125" customWidth="1"/>
+    <col min="6" max="6" width="67.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -383,15 +434,15 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:5">
       <c r="A2" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C2" s="1">
-        <v>20.0</v>
+        <v>20</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>6</v>
@@ -400,15 +451,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:5">
       <c r="A3" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C3" s="1">
-        <v>30.0</v>
+        <v>30</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>6</v>
@@ -417,15 +468,15 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:5">
       <c r="A4" s="1">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C4" s="1">
-        <v>15.0</v>
+        <v>15</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>9</v>
@@ -434,15 +485,15 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:5">
       <c r="A5" s="1">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C5" s="1">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>9</v>
@@ -451,15 +502,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:5">
       <c r="A6" s="1">
-        <v>6.0</v>
+        <v>6</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C6" s="1">
-        <v>30.0</v>
+        <v>30</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>9</v>
@@ -468,15 +519,15 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:5">
       <c r="A7" s="1">
-        <v>7.0</v>
+        <v>7</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C7" s="1">
-        <v>20.0</v>
+        <v>20</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>9</v>
@@ -485,15 +536,15 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:5">
       <c r="A8" s="1">
-        <v>8.0</v>
+        <v>8</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C8" s="1">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>6</v>
@@ -502,15 +553,15 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:5">
       <c r="A9" s="1">
-        <v>9.0</v>
+        <v>9</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C9" s="1">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>9</v>
@@ -519,15 +570,15 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:5">
       <c r="A10" s="1">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C10" s="1">
-        <v>30.0</v>
+        <v>30</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>9</v>
@@ -536,15 +587,15 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:5">
       <c r="A11" s="1">
-        <v>11.0</v>
+        <v>11</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C11" s="1">
-        <v>25.0</v>
+        <v>25</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>9</v>
@@ -553,15 +604,15 @@
         <v>17</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:5">
       <c r="A12" s="1">
-        <v>12.0</v>
+        <v>12</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C12" s="1">
-        <v>20.0</v>
+        <v>20</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>9</v>
@@ -570,15 +621,15 @@
         <v>18</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:5">
       <c r="A13" s="1">
-        <v>13.0</v>
+        <v>13</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C13" s="1">
-        <v>50.0</v>
+        <v>50</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>9</v>
@@ -587,15 +638,15 @@
         <v>19</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:5">
       <c r="A14" s="1">
-        <v>14.0</v>
+        <v>14</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C14" s="1">
-        <v>35.0</v>
+        <v>35</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>9</v>
@@ -604,15 +655,15 @@
         <v>20</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:5">
       <c r="A15" s="1">
-        <v>15.0</v>
+        <v>15</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C15" s="1">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>9</v>
@@ -621,15 +672,15 @@
         <v>21</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:5">
       <c r="A16" s="1">
-        <v>19.0</v>
+        <v>19</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C16" s="1">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>9</v>
@@ -638,15 +689,15 @@
         <v>22</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:5">
       <c r="A17" s="1">
-        <v>20.0</v>
+        <v>20</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C17" s="1">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>9</v>
@@ -655,15 +706,15 @@
         <v>23</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:5">
       <c r="A18" s="1">
-        <v>21.0</v>
+        <v>21</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C18" s="1">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>9</v>
@@ -672,15 +723,15 @@
         <v>24</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:5">
       <c r="A19" s="1">
-        <v>23.0</v>
+        <v>23</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C19" s="1">
-        <v>65.0</v>
+        <v>65</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>9</v>
@@ -689,15 +740,15 @@
         <v>25</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:5">
       <c r="A20" s="1">
-        <v>24.0</v>
+        <v>24</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C20" s="1">
-        <v>65.0</v>
+        <v>65</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>9</v>
@@ -706,15 +757,15 @@
         <v>26</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:5">
       <c r="A21" s="1">
-        <v>25.0</v>
+        <v>25</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C21" s="1">
-        <v>75.0</v>
+        <v>75</v>
       </c>
       <c r="D21" s="1" t="s">
         <v>6</v>
@@ -723,15 +774,15 @@
         <v>27</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:5">
       <c r="A22" s="1">
-        <v>26.0</v>
+        <v>26</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C22" s="1">
-        <v>70.0</v>
+        <v>70</v>
       </c>
       <c r="D22" s="1" t="s">
         <v>6</v>
@@ -740,15 +791,15 @@
         <v>28</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:5">
       <c r="A23" s="1">
-        <v>27.0</v>
+        <v>27</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C23" s="1">
-        <v>65.0</v>
+        <v>65</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>9</v>
@@ -757,15 +808,15 @@
         <v>29</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:5" ht="13.8" thickBot="1">
       <c r="A24" s="1">
-        <v>28.0</v>
+        <v>28</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C24" s="1">
-        <v>70.0</v>
+        <v>70</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>9</v>
@@ -774,7 +825,25 @@
         <v>30</v>
       </c>
     </row>
+    <row r="25" spans="1:5" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A25" s="2">
+        <v>29</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C25" s="1">
+        <v>200</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E25" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: implement listing automation suite including validation, mass deletion, and scheduling utilities
</commit_message>
<xml_diff>
--- a/data/data.xlsx
+++ b/data/data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Gathan\My Project\MacroListing\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98A5079F-7898-4FA5-8612-685700201418}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CCBA320-4935-4D27-8830-2A07CBB3B5A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2904" yWindow="1020" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet4" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="40">
   <si>
     <t>No</t>
   </si>
@@ -119,6 +119,27 @@
   </si>
   <si>
     <t>Asia | 64 Character(Inc Dupe) and 27 Lightcone | Casto E2 | Rate On Pity 40</t>
+  </si>
+  <si>
+    <t>wuthering waves</t>
+  </si>
+  <si>
+    <t>SEA</t>
+  </si>
+  <si>
+    <t>SEA | Qingxiao,Aemeath,Cartethyia,Mornye,Sigrika,Rebecca,Lupa,Ciaccona,Chisa,Shorekeeper,Phrolova,Jiyan,Cantarella,Yinlin | 8 Weapon Signature | Mid Explore | EndGame lvl 80</t>
+  </si>
+  <si>
+    <t>gender</t>
+  </si>
+  <si>
+    <t>Male</t>
+  </si>
+  <si>
+    <t>Asia | Dahlia E2,Firefly E2,Mortenax E2 and 18 Character 5 Star | 5 Lightcone Limited | EndGame Full Star</t>
+  </si>
+  <si>
+    <t>Asia | 33 Character 5 Star(Inc Dupe) and 20 Lightcone | Hyacine and Anaxa E1 | Pity Character 40 and Pity Lightcone 50</t>
   </si>
 </sst>
 </file>
@@ -180,7 +201,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -190,6 +211,7 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -408,7 +430,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="2" max="2" width="25.21875" customWidth="1"/>
@@ -417,7 +439,7 @@
     <col min="6" max="6" width="67.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:6" ht="13.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -433,8 +455,11 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5">
+      <c r="F1" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="13.2">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -451,7 +476,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:6" ht="13.2">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -468,7 +493,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:6" ht="13.2">
       <c r="A4" s="1">
         <v>4</v>
       </c>
@@ -485,7 +510,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:6" ht="13.2">
       <c r="A5" s="1">
         <v>5</v>
       </c>
@@ -502,7 +527,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:6" ht="13.2">
       <c r="A6" s="1">
         <v>6</v>
       </c>
@@ -519,7 +544,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:6" ht="13.2">
       <c r="A7" s="1">
         <v>7</v>
       </c>
@@ -536,7 +561,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:6" ht="13.2">
       <c r="A8" s="1">
         <v>8</v>
       </c>
@@ -553,7 +578,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:6" ht="13.2">
       <c r="A9" s="1">
         <v>9</v>
       </c>
@@ -570,7 +595,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:6" ht="13.2">
       <c r="A10" s="1">
         <v>10</v>
       </c>
@@ -587,7 +612,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
+    <row r="11" spans="1:6" ht="13.2">
       <c r="A11" s="1">
         <v>11</v>
       </c>
@@ -604,7 +629,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:5">
+    <row r="12" spans="1:6" ht="13.2">
       <c r="A12" s="1">
         <v>12</v>
       </c>
@@ -621,7 +646,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="13" spans="1:5">
+    <row r="13" spans="1:6" ht="13.2">
       <c r="A13" s="1">
         <v>13</v>
       </c>
@@ -638,7 +663,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="14" spans="1:5">
+    <row r="14" spans="1:6" ht="13.2">
       <c r="A14" s="1">
         <v>14</v>
       </c>
@@ -655,7 +680,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="1:5">
+    <row r="15" spans="1:6" ht="13.2">
       <c r="A15" s="1">
         <v>15</v>
       </c>
@@ -672,7 +697,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="16" spans="1:5">
+    <row r="16" spans="1:6" ht="13.2">
       <c r="A16" s="1">
         <v>19</v>
       </c>
@@ -689,7 +714,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="17" spans="1:5">
+    <row r="17" spans="1:6" ht="13.2">
       <c r="A17" s="1">
         <v>20</v>
       </c>
@@ -706,7 +731,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="18" spans="1:5">
+    <row r="18" spans="1:6" ht="13.2">
       <c r="A18" s="1">
         <v>21</v>
       </c>
@@ -723,7 +748,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="19" spans="1:5">
+    <row r="19" spans="1:6" ht="13.2">
       <c r="A19" s="1">
         <v>23</v>
       </c>
@@ -740,7 +765,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="20" spans="1:5">
+    <row r="20" spans="1:6" ht="13.2">
       <c r="A20" s="1">
         <v>24</v>
       </c>
@@ -757,7 +782,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="21" spans="1:5">
+    <row r="21" spans="1:6" ht="13.2">
       <c r="A21" s="1">
         <v>25</v>
       </c>
@@ -774,7 +799,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="22" spans="1:5">
+    <row r="22" spans="1:6" ht="13.2">
       <c r="A22" s="1">
         <v>26</v>
       </c>
@@ -791,7 +816,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="23" spans="1:5">
+    <row r="23" spans="1:6" ht="13.2">
       <c r="A23" s="1">
         <v>27</v>
       </c>
@@ -808,7 +833,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="24" spans="1:5" ht="13.8" thickBot="1">
+    <row r="24" spans="1:6" ht="13.8" thickBot="1">
       <c r="A24" s="1">
         <v>28</v>
       </c>
@@ -825,7 +850,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="25" spans="1:5" ht="15.75" customHeight="1" thickBot="1">
+    <row r="25" spans="1:6" ht="15.75" customHeight="1" thickBot="1">
       <c r="A25" s="2">
         <v>29</v>
       </c>
@@ -840,6 +865,60 @@
       </c>
       <c r="E25" s="4" t="s">
         <v>32</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="15.75" customHeight="1">
+      <c r="A26" s="1">
+        <v>30</v>
+      </c>
+      <c r="B26" t="s">
+        <v>33</v>
+      </c>
+      <c r="C26" s="1">
+        <v>70</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="15.75" customHeight="1">
+      <c r="A27" s="5">
+        <v>31</v>
+      </c>
+      <c r="B27" t="s">
+        <v>31</v>
+      </c>
+      <c r="C27" s="5">
+        <v>50</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="15.75" customHeight="1">
+      <c r="A28" s="5">
+        <v>32</v>
+      </c>
+      <c r="B28" t="s">
+        <v>31</v>
+      </c>
+      <c r="C28" s="5">
+        <v>50</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: implement automation framework for browser management and dynamic form interaction via Playwright
</commit_message>
<xml_diff>
--- a/data/data.xlsx
+++ b/data/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Gathan\My Project\MacroListing\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CCBA320-4935-4D27-8830-2A07CBB3B5A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFE50816-713E-4809-84F2-C7AC102EEC4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="42">
   <si>
     <t>No</t>
   </si>
@@ -140,6 +140,12 @@
   </si>
   <si>
     <t>Asia | 33 Character 5 Star(Inc Dupe) and 20 Lightcone | Hyacine and Anaxa E1 | Pity Character 40 and Pity Lightcone 50</t>
+  </si>
+  <si>
+    <t>Asia | 38 Character 5 Star and 30 Lightcone | Fugue and Huohuo E1 | 40 Ticket</t>
+  </si>
+  <si>
+    <t>Asia | 42 Character 5 Star and 16 Lightcone | E2 RuanMei and E1 Huohuo | Rate On 12 Ticket</t>
   </si>
 </sst>
 </file>
@@ -430,7 +436,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="2" max="2" width="25.21875" customWidth="1"/>
@@ -888,13 +894,13 @@
       </c>
     </row>
     <row r="27" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A27" s="5">
+      <c r="A27" s="1">
         <v>31</v>
       </c>
       <c r="B27" t="s">
         <v>31</v>
       </c>
-      <c r="C27" s="5">
+      <c r="C27" s="1">
         <v>50</v>
       </c>
       <c r="D27" s="1" t="s">
@@ -905,13 +911,13 @@
       </c>
     </row>
     <row r="28" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A28" s="5">
+      <c r="A28" s="1">
         <v>32</v>
       </c>
       <c r="B28" t="s">
         <v>31</v>
       </c>
-      <c r="C28" s="5">
+      <c r="C28" s="1">
         <v>50</v>
       </c>
       <c r="D28" s="1" t="s">
@@ -919,6 +925,40 @@
       </c>
       <c r="E28" s="4" t="s">
         <v>39</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="15.75" customHeight="1">
+      <c r="A29" s="5">
+        <v>33</v>
+      </c>
+      <c r="B29" t="s">
+        <v>31</v>
+      </c>
+      <c r="C29" s="5">
+        <v>100</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="15.75" customHeight="1">
+      <c r="A30" s="5">
+        <v>34</v>
+      </c>
+      <c r="B30" t="s">
+        <v>31</v>
+      </c>
+      <c r="C30" s="5">
+        <v>80</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>